<commit_message>
MyWebsite module - retry logic added for add projects
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/Modules/09_MyWebSite/MyWebSite/01_WebSite_Add.xlsx
+++ b/src/test/resources/testdata/Modules/09_MyWebSite/MyWebSite/01_WebSite_Add.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\testing\Documents\Bandhan_World_APPIUM\src\test\resources\testdata\Modules\09_MyWebSite\MyWebSite\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A43FA8A-806C-4F43-A98C-98DB2A5C5D5D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1DC081ED-98F9-46F8-80B9-4497FEB12050}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{D5674106-8292-4F40-9DFC-E6EAC771FC2F}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="1" xr2:uid="{D5674106-8292-4F40-9DFC-E6EAC771FC2F}"/>
   </bookViews>
   <sheets>
     <sheet name="TestCases" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2260" uniqueCount="552">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2260" uniqueCount="553">
   <si>
     <t>TESTCASE_ID</t>
   </si>
@@ -10588,6 +10588,12 @@
 clickon_nextbtn
 clickon_nextbtn
 verify_alert_dialog_title</t>
+  </si>
+  <si>
+    <t>project_add_projects
+project_clickon_submitbtn
+project_clickon_submitbtn
+verify_alert_dialog_title_retry</t>
   </si>
 </sst>
 </file>
@@ -15925,7 +15931,7 @@
         <v>265</v>
       </c>
       <c r="E141" s="6" t="s">
-        <v>549</v>
+        <v>552</v>
       </c>
       <c r="F141" s="1"/>
       <c r="G141" s="1"/>

</xml_diff>